<commit_message>
nuclear low utilization limit should not be zero
for some regions
</commit_message>
<xml_diff>
--- a/SuppXLS/Scen_dem-Base_KS_setup.xlsx
+++ b/SuppXLS/Scen_dem-Base_KS_setup.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="18350" windowHeight="8710" firstSheet="2" activeTab="2"/>
+    <workbookView windowWidth="18350" windowHeight="8710" firstSheet="2" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet name="Constants" sheetId="12" r:id="rId1"/>
@@ -90,6 +90,38 @@
 </file>
 
 <file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>xli9</author>
+  </authors>
+  <commentList>
+    <comment ref="A36" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t>xli9:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t xml:space="preserve">
+original Amit’s version is vacant/empty, then some nclear can have ca[acity but zero activity, that is not reasonable so we set as 0.1</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments4.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>xli9</author>
@@ -1562,12 +1594,12 @@
       <charset val="134"/>
     </font>
     <font>
+      <b/>
       <sz val="9"/>
       <name val="Times New Roman"/>
       <charset val="0"/>
     </font>
     <font>
-      <b/>
       <sz val="9"/>
       <name val="Times New Roman"/>
       <charset val="0"/>
@@ -26721,6 +26753,9 @@
       </c>
     </row>
     <row r="36" spans="1:46">
+      <c r="A36" s="2">
+        <v>0.1</v>
+      </c>
       <c r="B36" t="str">
         <f t="shared" si="15"/>
         <v>UCE_utilization_nuclear_LO</v>
@@ -26755,31 +26790,31 @@
       </c>
       <c r="J36" s="16">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>-0.0537</v>
       </c>
       <c r="K36" s="16">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>-0.08</v>
       </c>
       <c r="L36" s="16">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>-0.072</v>
       </c>
       <c r="M36" s="16">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>-0.08</v>
       </c>
       <c r="N36" s="16">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>-0.0712</v>
       </c>
       <c r="O36" s="16">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>-0.0548</v>
       </c>
       <c r="P36" s="16">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>-0.08</v>
       </c>
       <c r="Q36" s="16" t="str">
         <f t="shared" si="17"/>
@@ -26787,7 +26822,7 @@
       </c>
       <c r="R36" s="16">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>-0.08</v>
       </c>
       <c r="S36" s="16" t="str">
         <f t="shared" si="17"/>
@@ -26795,7 +26830,7 @@
       </c>
       <c r="T36" s="16">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>-0.063</v>
       </c>
       <c r="U36" s="16" t="str">
         <f t="shared" si="17"/>
@@ -26811,15 +26846,15 @@
       </c>
       <c r="X36" s="16">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>-0.0397</v>
       </c>
       <c r="Y36" s="16">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>-0.0377</v>
       </c>
       <c r="Z36" s="16">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>-0.08</v>
       </c>
       <c r="AA36" s="16" t="str">
         <f t="shared" si="17"/>
@@ -26831,11 +26866,11 @@
       </c>
       <c r="AC36" s="16">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>-0.0705</v>
       </c>
       <c r="AD36" s="16">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>-0.0786</v>
       </c>
       <c r="AE36" s="16" t="str">
         <f t="shared" si="17"/>
@@ -26843,19 +26878,19 @@
       </c>
       <c r="AF36" s="16">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>-0.0526</v>
       </c>
       <c r="AG36" s="16">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>-0.08</v>
       </c>
       <c r="AH36" s="16">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>-0.073</v>
       </c>
       <c r="AI36" s="16">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>-0.0699</v>
       </c>
       <c r="AJ36" s="16" t="str">
         <f t="shared" si="13"/>
@@ -26863,11 +26898,11 @@
       </c>
       <c r="AK36" s="16">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>-0.062</v>
       </c>
       <c r="AL36" s="16">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>-0.0512</v>
       </c>
       <c r="AM36" s="16" t="str">
         <f t="shared" si="13"/>
@@ -26886,6 +26921,9 @@
       </c>
     </row>
     <row r="37" spans="1:46">
+      <c r="A37" s="2">
+        <v>0.1</v>
+      </c>
       <c r="B37" t="str">
         <f t="shared" si="15"/>
         <v>UCE_utilization_oil_\I: LO</v>
@@ -26900,59 +26938,59 @@
       </c>
       <c r="E37" s="16">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>-0.0367</v>
       </c>
       <c r="F37" s="16">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>-0.0146</v>
       </c>
       <c r="G37" s="16">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>-0.021</v>
       </c>
       <c r="H37" s="16">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>-0.0463</v>
       </c>
       <c r="I37" s="16">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>-0.021</v>
       </c>
       <c r="J37" s="16">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>-0.08</v>
       </c>
       <c r="K37" s="16">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>-0.016</v>
       </c>
       <c r="L37" s="16">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>-0.052</v>
       </c>
       <c r="M37" s="16">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>-0.0003</v>
       </c>
       <c r="N37" s="16">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>-0.08</v>
       </c>
       <c r="O37" s="16">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>-0.0571</v>
       </c>
       <c r="P37" s="16">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>-0.08</v>
       </c>
       <c r="Q37" s="16">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>-0.0301</v>
       </c>
       <c r="R37" s="16">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>-0.007</v>
       </c>
       <c r="S37" s="16">
         <f t="shared" si="17"/>
@@ -26960,83 +26998,83 @@
       </c>
       <c r="T37" s="16">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>-0.0021</v>
       </c>
       <c r="U37" s="16">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>-0.0111</v>
       </c>
       <c r="V37" s="16">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>-0.0782</v>
       </c>
       <c r="W37" s="16">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>-0.0089</v>
       </c>
       <c r="X37" s="16">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>-0.0221</v>
       </c>
       <c r="Y37" s="16">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>-0.0616</v>
       </c>
       <c r="Z37" s="16">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>-0.0117</v>
       </c>
       <c r="AA37" s="16">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>-0.0632</v>
       </c>
       <c r="AB37" s="16">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>-0.08</v>
       </c>
       <c r="AC37" s="16">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>-0.02</v>
       </c>
       <c r="AD37" s="16">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>-0.08</v>
       </c>
       <c r="AE37" s="16">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>-0.0629</v>
       </c>
       <c r="AF37" s="16">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>-0.0001</v>
       </c>
       <c r="AG37" s="16">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>-0.0374</v>
       </c>
       <c r="AH37" s="16">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>-0.01</v>
       </c>
       <c r="AI37" s="16">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>-0.026</v>
       </c>
       <c r="AJ37" s="16">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>-0.0059</v>
       </c>
       <c r="AK37" s="16">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>-0.022</v>
       </c>
       <c r="AL37" s="16">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>-0.08</v>
       </c>
       <c r="AM37" s="16">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>-0.0103</v>
       </c>
       <c r="AO37" s="16" t="str">
         <f t="shared" si="18"/>
@@ -27051,6 +27089,9 @@
       </c>
     </row>
     <row r="38" spans="1:46">
+      <c r="A38" s="2">
+        <v>0.1</v>
+      </c>
       <c r="B38" t="str">
         <f t="shared" si="15"/>
         <v>UCE_utilization_bioenergy_UP</v>
@@ -27216,6 +27257,9 @@
       </c>
     </row>
     <row r="39" spans="1:46">
+      <c r="A39" s="2">
+        <v>0.1</v>
+      </c>
       <c r="B39" t="str">
         <f t="shared" si="15"/>
         <v>UCE_utilization_coal_UP</v>
@@ -27887,6 +27931,7 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
FIX NUCLEAR util rate
</commit_message>
<xml_diff>
--- a/SuppXLS/Scen_dem-Base_KS_setup.xlsx
+++ b/SuppXLS/Scen_dem-Base_KS_setup.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="18350" windowHeight="8710" firstSheet="2" activeTab="2"/>
+    <workbookView windowWidth="18350" windowHeight="8710" firstSheet="2" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet name="Constants" sheetId="12" r:id="rId1"/>
@@ -90,38 +90,6 @@
 </file>
 
 <file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>xli9</author>
-  </authors>
-  <commentList>
-    <comment ref="A36" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <rFont val="Times New Roman"/>
-            <charset val="0"/>
-          </rPr>
-          <t>xli9:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <rFont val="Times New Roman"/>
-            <charset val="0"/>
-          </rPr>
-          <t xml:space="preserve">
-original Amit’s version is vacant/empty, then some nclear can have ca[acity but zero activity, that is not reasonable so we set as 0.1</t>
-        </r>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments4.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>xli9</author>
@@ -1597,18 +1565,18 @@
       <b/>
       <sz val="9"/>
       <name val="Times New Roman"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
-      <name val="Times New Roman"/>
       <charset val="0"/>
     </font>
     <font>
       <sz val="9"/>
       <name val="Times New Roman"/>
       <charset val="0"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <name val="Times New Roman"/>
+      <charset val="134"/>
     </font>
     <font>
       <sz val="9"/>
@@ -26264,139 +26232,139 @@
         <v>-0.0042</v>
       </c>
       <c r="F33" s="16">
-        <f t="shared" ref="F33:AM37" si="13">IF(F7="","",-MIN(F7,F2,0.8)*$A33)</f>
+        <f>IF(F7="","",-MIN(F7,F2,0.8)*$A33)</f>
         <v>-0.0525</v>
       </c>
       <c r="G33" s="16">
-        <f t="shared" si="13"/>
+        <f>IF(G7="","",-MIN(G7,G2,0.8)*$A33)</f>
         <v>-0.1218</v>
       </c>
       <c r="H33" s="16">
-        <f t="shared" si="13"/>
+        <f>IF(H7="","",-MIN(H7,H2,0.8)*$A33)</f>
         <v>-0.1287</v>
       </c>
       <c r="I33" s="16">
-        <f t="shared" si="13"/>
+        <f>IF(I7="","",-MIN(I7,I2,0.8)*$A33)</f>
         <v>-0.1668</v>
       </c>
       <c r="J33" s="16">
-        <f t="shared" si="13"/>
+        <f>IF(J7="","",-MIN(J7,J2,0.8)*$A33)</f>
         <v>-0.24</v>
       </c>
       <c r="K33" s="16">
-        <f t="shared" si="13"/>
+        <f>IF(K7="","",-MIN(K7,K2,0.8)*$A33)</f>
         <v>-0.1089</v>
       </c>
       <c r="L33" s="16">
-        <f t="shared" si="13"/>
+        <f>IF(L7="","",-MIN(L7,L2,0.8)*$A33)</f>
         <v>-0.24</v>
       </c>
       <c r="M33" s="16">
-        <f t="shared" si="13"/>
+        <f>IF(M7="","",-MIN(M7,M2,0.8)*$A33)</f>
         <v>-0.165</v>
       </c>
       <c r="N33" s="16">
-        <f t="shared" si="13"/>
+        <f>IF(N7="","",-MIN(N7,N2,0.8)*$A33)</f>
         <v>-0.2106</v>
       </c>
       <c r="O33" s="16">
-        <f t="shared" si="13"/>
+        <f>IF(O7="","",-MIN(O7,O2,0.8)*$A33)</f>
         <v>-0.2085</v>
       </c>
       <c r="P33" s="16">
-        <f t="shared" si="13"/>
+        <f>IF(P7="","",-MIN(P7,P2,0.8)*$A33)</f>
         <v>-0.1767</v>
       </c>
       <c r="Q33" s="16">
-        <f t="shared" si="13"/>
+        <f>IF(Q7="","",-MIN(Q7,Q2,0.8)*$A33)</f>
         <v>-0.1407</v>
       </c>
       <c r="R33" s="16">
-        <f t="shared" si="13"/>
+        <f>IF(R7="","",-MIN(R7,R2,0.8)*$A33)</f>
         <v>-0.1467</v>
       </c>
       <c r="S33" s="16" t="str">
-        <f t="shared" si="13"/>
+        <f>IF(S7="","",-MIN(S7,S2,0.8)*$A33)</f>
         <v/>
       </c>
       <c r="T33" s="16">
-        <f t="shared" si="13"/>
+        <f>IF(T7="","",-MIN(T7,T2,0.8)*$A33)</f>
         <v>-0.0921</v>
       </c>
       <c r="U33" s="16">
-        <f t="shared" si="13"/>
+        <f>IF(U7="","",-MIN(U7,U2,0.8)*$A33)</f>
         <v>-0.24</v>
       </c>
       <c r="V33" s="16">
-        <f t="shared" si="13"/>
+        <f>IF(V7="","",-MIN(V7,V2,0.8)*$A33)</f>
         <v>-0.1872</v>
       </c>
       <c r="W33" s="16">
-        <f t="shared" si="13"/>
+        <f>IF(W7="","",-MIN(W7,W2,0.8)*$A33)</f>
         <v>-0.24</v>
       </c>
       <c r="X33" s="16">
-        <f t="shared" si="13"/>
+        <f>IF(X7="","",-MIN(X7,X2,0.8)*$A33)</f>
         <v>-0.1044</v>
       </c>
       <c r="Y33" s="16">
-        <f t="shared" si="13"/>
+        <f>IF(Y7="","",-MIN(Y7,Y2,0.8)*$A33)</f>
         <v>-0.0882</v>
       </c>
       <c r="Z33" s="16">
-        <f t="shared" si="13"/>
+        <f>IF(Z7="","",-MIN(Z7,Z2,0.8)*$A33)</f>
         <v>-0.1641</v>
       </c>
       <c r="AA33" s="16">
-        <f t="shared" si="13"/>
+        <f>IF(AA7="","",-MIN(AA7,AA2,0.8)*$A33)</f>
         <v>-0.0855</v>
       </c>
       <c r="AB33" s="16">
-        <f t="shared" si="13"/>
+        <f>IF(AB7="","",-MIN(AB7,AB2,0.8)*$A33)</f>
         <v>-0.2232</v>
       </c>
       <c r="AC33" s="16">
-        <f t="shared" si="13"/>
+        <f>IF(AC7="","",-MIN(AC7,AC2,0.8)*$A33)</f>
         <v>-0.1248</v>
       </c>
       <c r="AD33" s="16">
-        <f t="shared" si="13"/>
+        <f>IF(AD7="","",-MIN(AD7,AD2,0.8)*$A33)</f>
         <v>-0.0153</v>
       </c>
       <c r="AE33" s="16" t="str">
-        <f t="shared" si="13"/>
+        <f>IF(AE7="","",-MIN(AE7,AE2,0.8)*$A33)</f>
         <v/>
       </c>
       <c r="AF33" s="16">
-        <f t="shared" si="13"/>
+        <f>IF(AF7="","",-MIN(AF7,AF2,0.8)*$A33)</f>
         <v>-0.0435</v>
       </c>
       <c r="AG33" s="16">
-        <f t="shared" si="13"/>
+        <f>IF(AG7="","",-MIN(AG7,AG2,0.8)*$A33)</f>
         <v>-0.1812</v>
       </c>
       <c r="AH33" s="16">
-        <f t="shared" si="13"/>
+        <f>IF(AH7="","",-MIN(AH7,AH2,0.8)*$A33)</f>
         <v>-0.1155</v>
       </c>
       <c r="AI33" s="16">
-        <f t="shared" si="13"/>
+        <f>IF(AI7="","",-MIN(AI7,AI2,0.8)*$A33)</f>
         <v>-0.24</v>
       </c>
       <c r="AJ33" s="16">
-        <f t="shared" si="13"/>
+        <f>IF(AJ7="","",-MIN(AJ7,AJ2,0.8)*$A33)</f>
         <v>-0.135</v>
       </c>
       <c r="AK33" s="16">
-        <f t="shared" si="13"/>
+        <f>IF(AK7="","",-MIN(AK7,AK2,0.8)*$A33)</f>
         <v>-0.1737</v>
       </c>
       <c r="AL33" s="16">
-        <f t="shared" si="13"/>
+        <f>IF(AL7="","",-MIN(AL7,AL2,0.8)*$A33)</f>
         <v>-0.0513</v>
       </c>
       <c r="AM33" s="16">
-        <f t="shared" si="13"/>
+        <f>IF(AM7="","",-MIN(AM7,AM2,0.8)*$A33)</f>
         <v>-0.0684</v>
       </c>
       <c r="AO33" s="16" t="str">
@@ -26404,7 +26372,7 @@
         <v>ELE,CHP</v>
       </c>
       <c r="AP33" s="16" t="str">
-        <f t="shared" ref="AP33:AP42" si="14">AP22</f>
+        <f t="shared" ref="AP33:AP42" si="13">AP22</f>
         <v>elcbsl,indbio</v>
       </c>
       <c r="AR33" s="43" t="s">
@@ -26416,163 +26384,163 @@
         <v>0.3</v>
       </c>
       <c r="B34" t="str">
-        <f t="shared" ref="B34:C42" si="15">B23</f>
+        <f t="shared" ref="B34:C42" si="14">B23</f>
         <v>UCE_utilization_coal_LO</v>
       </c>
       <c r="C34" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="14"/>
         <v>LO</v>
       </c>
       <c r="D34">
-        <f t="shared" ref="D34:D42" si="16">D23+7</f>
+        <f t="shared" ref="D34:D42" si="15">D23+7</f>
         <v>2030</v>
       </c>
       <c r="E34" s="16">
-        <f t="shared" ref="E34:AG37" si="17">IF(E8="","",-MIN(E8,E3,0.8)*$A34)</f>
+        <f t="shared" ref="E34:AG37" si="16">IF(E8="","",-MIN(E8,E3,0.8)*$A34)</f>
         <v>-0.171</v>
       </c>
       <c r="F34" s="16">
-        <f t="shared" si="17"/>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="G34" s="16">
-        <f t="shared" si="17"/>
+        <f t="shared" si="16"/>
         <v>-0.1815</v>
       </c>
       <c r="H34" s="16">
-        <f t="shared" si="17"/>
+        <f t="shared" si="16"/>
         <v>-0.0831</v>
       </c>
       <c r="I34" s="16">
-        <f t="shared" si="17"/>
+        <f t="shared" si="16"/>
         <v>-0.24</v>
       </c>
       <c r="J34" s="16">
-        <f t="shared" si="17"/>
+        <f t="shared" si="16"/>
         <v>-0.0753</v>
       </c>
       <c r="K34" s="16">
-        <f t="shared" si="17"/>
+        <f t="shared" si="16"/>
         <v>-0.1527</v>
       </c>
       <c r="L34" s="16">
-        <f t="shared" si="17"/>
+        <f t="shared" si="16"/>
         <v>-0.1545</v>
       </c>
       <c r="M34" s="16">
-        <f t="shared" si="17"/>
+        <f t="shared" si="16"/>
         <v>-0.1104</v>
       </c>
       <c r="N34" s="16">
-        <f t="shared" si="17"/>
+        <f t="shared" si="16"/>
         <v>-0.1284</v>
       </c>
       <c r="O34" s="16">
-        <f t="shared" si="17"/>
+        <f t="shared" si="16"/>
         <v>-0.0282</v>
       </c>
       <c r="P34" s="16">
-        <f t="shared" si="17"/>
+        <f t="shared" si="16"/>
         <v>-0.0984</v>
       </c>
       <c r="Q34" s="16">
-        <f t="shared" si="17"/>
+        <f t="shared" si="16"/>
         <v>-0.0561</v>
       </c>
       <c r="R34" s="16">
-        <f t="shared" si="17"/>
+        <f t="shared" si="16"/>
         <v>-0.0804</v>
       </c>
       <c r="S34" s="16" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="T34" s="16">
-        <f t="shared" si="17"/>
+        <f t="shared" si="16"/>
         <v>-0.1734</v>
       </c>
       <c r="U34" s="16">
-        <f t="shared" si="17"/>
+        <f t="shared" si="16"/>
         <v>-0.0189</v>
       </c>
       <c r="V34" s="16">
-        <f t="shared" si="17"/>
+        <f t="shared" si="16"/>
         <v>-0.0591</v>
       </c>
       <c r="W34" s="16">
-        <f t="shared" si="17"/>
+        <f t="shared" si="16"/>
         <v>-0.2022</v>
       </c>
       <c r="X34" s="16">
-        <f t="shared" si="17"/>
+        <f t="shared" si="16"/>
         <v>-0.1494</v>
       </c>
       <c r="Y34" s="16">
-        <f t="shared" si="17"/>
+        <f t="shared" si="16"/>
         <v>-0.1155</v>
       </c>
       <c r="Z34" s="16">
-        <f t="shared" si="17"/>
+        <f t="shared" si="16"/>
         <v>-0.1152</v>
       </c>
       <c r="AA34" s="16">
-        <f t="shared" si="17"/>
+        <f t="shared" si="16"/>
         <v>-0.24</v>
       </c>
       <c r="AB34" s="16">
-        <f t="shared" si="17"/>
+        <f t="shared" si="16"/>
         <v>-0.1236</v>
       </c>
       <c r="AC34" s="16">
-        <f t="shared" si="17"/>
+        <f t="shared" si="16"/>
         <v>-0.1671</v>
       </c>
       <c r="AD34" s="16">
-        <f t="shared" si="17"/>
+        <f t="shared" si="16"/>
         <v>-0.126</v>
       </c>
       <c r="AE34" s="16" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
       <c r="AF34" s="16">
-        <f t="shared" si="17"/>
+        <f t="shared" si="16"/>
         <v>-0.1422</v>
       </c>
       <c r="AG34" s="16">
-        <f t="shared" si="17"/>
+        <f t="shared" si="16"/>
         <v>-0.0375</v>
       </c>
       <c r="AH34" s="16">
+        <f>IF(AH8="","",-MIN(AH8,AH3,0.8)*$A34)</f>
+        <v>-0.0498</v>
+      </c>
+      <c r="AI34" s="16" t="str">
+        <f>IF(AI8="","",-MIN(AI8,AI3,0.8)*$A34)</f>
+        <v/>
+      </c>
+      <c r="AJ34" s="16">
+        <f>IF(AJ8="","",-MIN(AJ8,AJ3,0.8)*$A34)</f>
+        <v>-0.1704</v>
+      </c>
+      <c r="AK34" s="16">
+        <f>IF(AK8="","",-MIN(AK8,AK3,0.8)*$A34)</f>
+        <v>-0.0246</v>
+      </c>
+      <c r="AL34" s="16">
+        <f>IF(AL8="","",-MIN(AL8,AL3,0.8)*$A34)</f>
+        <v>0</v>
+      </c>
+      <c r="AM34" s="16">
+        <f>IF(AM8="","",-MIN(AM8,AM3,0.8)*$A34)</f>
+        <v>-0.177</v>
+      </c>
+      <c r="AO34" s="16" t="str">
+        <f t="shared" ref="AO34:AO42" si="17">AO23</f>
+        <v>ELE,CHP</v>
+      </c>
+      <c r="AP34" s="16" t="str">
         <f t="shared" si="13"/>
-        <v>-0.0498</v>
-      </c>
-      <c r="AI34" s="16" t="str">
-        <f t="shared" si="13"/>
-        <v/>
-      </c>
-      <c r="AJ34" s="16">
-        <f t="shared" si="13"/>
-        <v>-0.1704</v>
-      </c>
-      <c r="AK34" s="16">
-        <f t="shared" si="13"/>
-        <v>-0.0246</v>
-      </c>
-      <c r="AL34" s="16">
-        <f t="shared" si="13"/>
-        <v>0</v>
-      </c>
-      <c r="AM34" s="16">
-        <f t="shared" si="13"/>
-        <v>-0.177</v>
-      </c>
-      <c r="AO34" s="16" t="str">
-        <f t="shared" ref="AO34:AO42" si="18">AO23</f>
-        <v>ELE,CHP</v>
-      </c>
-      <c r="AP34" s="16" t="str">
-        <f t="shared" si="14"/>
         <v>???coa,elccob</v>
       </c>
       <c r="AR34" s="43" t="s">
@@ -26584,163 +26552,163 @@
         <v>0.3</v>
       </c>
       <c r="B35" t="str">
+        <f t="shared" si="14"/>
+        <v>UCE_utilization_gas_LO</v>
+      </c>
+      <c r="C35" t="str">
+        <f t="shared" si="14"/>
+        <v>LO</v>
+      </c>
+      <c r="D35">
         <f t="shared" si="15"/>
-        <v>UCE_utilization_gas_LO</v>
-      </c>
-      <c r="C35" t="str">
-        <f t="shared" si="15"/>
-        <v>LO</v>
-      </c>
-      <c r="D35">
+        <v>2030</v>
+      </c>
+      <c r="E35" s="16">
         <f t="shared" si="16"/>
-        <v>2030</v>
-      </c>
-      <c r="E35" s="16">
+        <v>-0.1119</v>
+      </c>
+      <c r="F35" s="16">
+        <f t="shared" si="16"/>
+        <v>-0.0954</v>
+      </c>
+      <c r="G35" s="16">
+        <f t="shared" si="16"/>
+        <v>-0.0591</v>
+      </c>
+      <c r="H35" s="16">
+        <f t="shared" si="16"/>
+        <v>-0.0381</v>
+      </c>
+      <c r="I35" s="16">
+        <f t="shared" si="16"/>
+        <v>-0.0189</v>
+      </c>
+      <c r="J35" s="16">
+        <f t="shared" si="16"/>
+        <v>-0.0936</v>
+      </c>
+      <c r="K35" s="16">
+        <f t="shared" si="16"/>
+        <v>-0.0696</v>
+      </c>
+      <c r="L35" s="16">
+        <f t="shared" si="16"/>
+        <v>-0.0777</v>
+      </c>
+      <c r="M35" s="16">
+        <f t="shared" si="16"/>
+        <v>-0.087</v>
+      </c>
+      <c r="N35" s="16">
+        <f t="shared" si="16"/>
+        <v>-0.0264</v>
+      </c>
+      <c r="O35" s="16">
+        <f t="shared" si="16"/>
+        <v>-0.0189</v>
+      </c>
+      <c r="P35" s="16">
+        <f t="shared" si="16"/>
+        <v>-0.0762</v>
+      </c>
+      <c r="Q35" s="16">
+        <f t="shared" si="16"/>
+        <v>-0.0462</v>
+      </c>
+      <c r="R35" s="16">
+        <f t="shared" si="16"/>
+        <v>-0.0492</v>
+      </c>
+      <c r="S35" s="16" t="str">
+        <f t="shared" si="16"/>
+        <v/>
+      </c>
+      <c r="T35" s="16">
+        <f t="shared" si="16"/>
+        <v>-0.0495</v>
+      </c>
+      <c r="U35" s="16">
+        <f t="shared" si="16"/>
+        <v>-0.0966</v>
+      </c>
+      <c r="V35" s="16">
+        <f t="shared" si="16"/>
+        <v>-0.0474</v>
+      </c>
+      <c r="W35" s="16">
+        <f t="shared" si="16"/>
+        <v>-0.1395</v>
+      </c>
+      <c r="X35" s="16">
+        <f t="shared" si="16"/>
+        <v>-0.1056</v>
+      </c>
+      <c r="Y35" s="16">
+        <f t="shared" si="16"/>
+        <v>-0.1167</v>
+      </c>
+      <c r="Z35" s="16">
+        <f t="shared" si="16"/>
+        <v>-0.0942</v>
+      </c>
+      <c r="AA35" s="16">
+        <f t="shared" si="16"/>
+        <v>-0.0138</v>
+      </c>
+      <c r="AB35" s="16">
+        <f t="shared" si="16"/>
+        <v>-0.1116</v>
+      </c>
+      <c r="AC35" s="16">
+        <f t="shared" si="16"/>
+        <v>-0.1371</v>
+      </c>
+      <c r="AD35" s="16">
+        <f t="shared" si="16"/>
+        <v>-0.1425</v>
+      </c>
+      <c r="AE35" s="16">
+        <f t="shared" si="16"/>
+        <v>-0.1158</v>
+      </c>
+      <c r="AF35" s="16">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="AG35" s="16">
+        <f t="shared" si="16"/>
+        <v>-0.0585</v>
+      </c>
+      <c r="AH35" s="16">
+        <f>IF(AH9="","",-MIN(AH9,AH4,0.8)*$A35)</f>
+        <v>-0.0144</v>
+      </c>
+      <c r="AI35" s="16">
+        <f>IF(AI9="","",-MIN(AI9,AI4,0.8)*$A35)</f>
+        <v>-0.0714</v>
+      </c>
+      <c r="AJ35" s="16">
+        <f>IF(AJ9="","",-MIN(AJ9,AJ4,0.8)*$A35)</f>
+        <v>-0.0681</v>
+      </c>
+      <c r="AK35" s="16">
+        <f>IF(AK9="","",-MIN(AK9,AK4,0.8)*$A35)</f>
+        <v>-0.0903</v>
+      </c>
+      <c r="AL35" s="16">
+        <f>IF(AL9="","",-MIN(AL9,AL4,0.8)*$A35)</f>
+        <v>-0.042</v>
+      </c>
+      <c r="AM35" s="16">
+        <f>IF(AM9="","",-MIN(AM9,AM4,0.8)*$A35)</f>
+        <v>-0.0186</v>
+      </c>
+      <c r="AO35" s="16" t="str">
         <f t="shared" si="17"/>
-        <v>-0.1119</v>
-      </c>
-      <c r="F35" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.0954</v>
-      </c>
-      <c r="G35" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.0591</v>
-      </c>
-      <c r="H35" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.0381</v>
-      </c>
-      <c r="I35" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.0189</v>
-      </c>
-      <c r="J35" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.0936</v>
-      </c>
-      <c r="K35" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.0696</v>
-      </c>
-      <c r="L35" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.0777</v>
-      </c>
-      <c r="M35" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.087</v>
-      </c>
-      <c r="N35" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.0264</v>
-      </c>
-      <c r="O35" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.0189</v>
-      </c>
-      <c r="P35" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.0762</v>
-      </c>
-      <c r="Q35" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.0462</v>
-      </c>
-      <c r="R35" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.0492</v>
-      </c>
-      <c r="S35" s="16" t="str">
-        <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="T35" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.0495</v>
-      </c>
-      <c r="U35" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.0966</v>
-      </c>
-      <c r="V35" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.0474</v>
-      </c>
-      <c r="W35" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.1395</v>
-      </c>
-      <c r="X35" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.1056</v>
-      </c>
-      <c r="Y35" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.1167</v>
-      </c>
-      <c r="Z35" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.0942</v>
-      </c>
-      <c r="AA35" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.0138</v>
-      </c>
-      <c r="AB35" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.1116</v>
-      </c>
-      <c r="AC35" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.1371</v>
-      </c>
-      <c r="AD35" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.1425</v>
-      </c>
-      <c r="AE35" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.1158</v>
-      </c>
-      <c r="AF35" s="16">
-        <f t="shared" si="17"/>
-        <v>0</v>
-      </c>
-      <c r="AG35" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.0585</v>
-      </c>
-      <c r="AH35" s="16">
+        <v>ELE,CHP</v>
+      </c>
+      <c r="AP35" s="16" t="str">
         <f t="shared" si="13"/>
-        <v>-0.0144</v>
-      </c>
-      <c r="AI35" s="16">
-        <f t="shared" si="13"/>
-        <v>-0.0714</v>
-      </c>
-      <c r="AJ35" s="16">
-        <f t="shared" si="13"/>
-        <v>-0.0681</v>
-      </c>
-      <c r="AK35" s="16">
-        <f t="shared" si="13"/>
-        <v>-0.0903</v>
-      </c>
-      <c r="AL35" s="16">
-        <f t="shared" si="13"/>
-        <v>-0.042</v>
-      </c>
-      <c r="AM35" s="16">
-        <f t="shared" si="13"/>
-        <v>-0.0186</v>
-      </c>
-      <c r="AO35" s="16" t="str">
-        <f t="shared" si="18"/>
-        <v>ELE,CHP</v>
-      </c>
-      <c r="AP35" s="16" t="str">
-        <f t="shared" si="14"/>
         <v>???nga</v>
       </c>
       <c r="AR35" s="43" t="s">
@@ -26754,167 +26722,60 @@
       </c>
     </row>
     <row r="36" spans="1:46">
-      <c r="A36" s="19">
-        <v>0.1</v>
-      </c>
+      <c r="A36" s="19"/>
       <c r="B36" t="str">
+        <f t="shared" si="14"/>
+        <v>UCE_utilization_nuclear_LO</v>
+      </c>
+      <c r="C36" t="str">
+        <f t="shared" si="14"/>
+        <v>LO</v>
+      </c>
+      <c r="D36">
         <f t="shared" si="15"/>
-        <v>UCE_utilization_nuclear_LO</v>
-      </c>
-      <c r="C36" t="str">
-        <f t="shared" si="15"/>
-        <v>LO</v>
-      </c>
-      <c r="D36">
-        <f t="shared" si="16"/>
         <v>2030</v>
       </c>
-      <c r="E36" s="16" t="str">
+      <c r="E36" s="16"/>
+      <c r="F36" s="16"/>
+      <c r="G36" s="16"/>
+      <c r="H36" s="16"/>
+      <c r="I36" s="16"/>
+      <c r="J36" s="16"/>
+      <c r="K36" s="16"/>
+      <c r="L36" s="16"/>
+      <c r="M36" s="16"/>
+      <c r="N36" s="16"/>
+      <c r="O36" s="16"/>
+      <c r="P36" s="16"/>
+      <c r="Q36" s="16"/>
+      <c r="R36" s="16"/>
+      <c r="S36" s="16"/>
+      <c r="T36" s="16"/>
+      <c r="U36" s="16"/>
+      <c r="V36" s="16"/>
+      <c r="W36" s="16"/>
+      <c r="X36" s="16"/>
+      <c r="Y36" s="16"/>
+      <c r="Z36" s="16"/>
+      <c r="AA36" s="16"/>
+      <c r="AB36" s="16"/>
+      <c r="AC36" s="16"/>
+      <c r="AD36" s="16"/>
+      <c r="AE36" s="16"/>
+      <c r="AF36" s="16"/>
+      <c r="AG36" s="16"/>
+      <c r="AH36" s="16"/>
+      <c r="AI36" s="16"/>
+      <c r="AJ36" s="16"/>
+      <c r="AK36" s="16"/>
+      <c r="AL36" s="16"/>
+      <c r="AM36" s="16"/>
+      <c r="AO36" s="16" t="str">
         <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="F36" s="16" t="str">
-        <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="G36" s="16" t="str">
-        <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="H36" s="16" t="str">
-        <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="I36" s="16" t="str">
-        <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="J36" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.0537</v>
-      </c>
-      <c r="K36" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.08</v>
-      </c>
-      <c r="L36" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.072</v>
-      </c>
-      <c r="M36" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.08</v>
-      </c>
-      <c r="N36" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.0712</v>
-      </c>
-      <c r="O36" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.0548</v>
-      </c>
-      <c r="P36" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.08</v>
-      </c>
-      <c r="Q36" s="16" t="str">
-        <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="R36" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.08</v>
-      </c>
-      <c r="S36" s="16" t="str">
-        <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="T36" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.063</v>
-      </c>
-      <c r="U36" s="16" t="str">
-        <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="V36" s="16" t="str">
-        <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="W36" s="16">
-        <f t="shared" si="17"/>
-        <v>0</v>
-      </c>
-      <c r="X36" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.0397</v>
-      </c>
-      <c r="Y36" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.0377</v>
-      </c>
-      <c r="Z36" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.08</v>
-      </c>
-      <c r="AA36" s="16" t="str">
-        <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="AB36" s="16" t="str">
-        <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="AC36" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.0705</v>
-      </c>
-      <c r="AD36" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.0786</v>
-      </c>
-      <c r="AE36" s="16" t="str">
-        <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="AF36" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.0526</v>
-      </c>
-      <c r="AG36" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.08</v>
-      </c>
-      <c r="AH36" s="16">
+        <v>ELE,CHP</v>
+      </c>
+      <c r="AP36" s="16" t="str">
         <f t="shared" si="13"/>
-        <v>-0.073</v>
-      </c>
-      <c r="AI36" s="16">
-        <f t="shared" si="13"/>
-        <v>-0.0699</v>
-      </c>
-      <c r="AJ36" s="16" t="str">
-        <f t="shared" si="13"/>
-        <v/>
-      </c>
-      <c r="AK36" s="16">
-        <f t="shared" si="13"/>
-        <v>-0.062</v>
-      </c>
-      <c r="AL36" s="16">
-        <f t="shared" si="13"/>
-        <v>-0.0512</v>
-      </c>
-      <c r="AM36" s="16" t="str">
-        <f t="shared" si="13"/>
-        <v/>
-      </c>
-      <c r="AO36" s="16" t="str">
-        <f t="shared" si="18"/>
-        <v>ELE,CHP</v>
-      </c>
-      <c r="AP36" s="16" t="str">
-        <f t="shared" si="14"/>
         <v>???nuc</v>
       </c>
       <c r="AR36" s="43" t="s">
@@ -26922,167 +26783,60 @@
       </c>
     </row>
     <row r="37" spans="1:46">
-      <c r="A37" s="19">
-        <v>0.1</v>
-      </c>
+      <c r="A37" s="19"/>
       <c r="B37" t="str">
+        <f t="shared" si="14"/>
+        <v>UCE_utilization_oil_\I: LO</v>
+      </c>
+      <c r="C37" t="str">
+        <f t="shared" si="14"/>
+        <v>\I: LO</v>
+      </c>
+      <c r="D37">
         <f t="shared" si="15"/>
-        <v>UCE_utilization_oil_\I: LO</v>
-      </c>
-      <c r="C37" t="str">
-        <f t="shared" si="15"/>
-        <v>\I: LO</v>
-      </c>
-      <c r="D37">
-        <f t="shared" si="16"/>
         <v>2030</v>
       </c>
-      <c r="E37" s="16">
+      <c r="E37" s="16"/>
+      <c r="F37" s="16"/>
+      <c r="G37" s="16"/>
+      <c r="H37" s="16"/>
+      <c r="I37" s="16"/>
+      <c r="J37" s="16"/>
+      <c r="K37" s="16"/>
+      <c r="L37" s="16"/>
+      <c r="M37" s="16"/>
+      <c r="N37" s="16"/>
+      <c r="O37" s="16"/>
+      <c r="P37" s="16"/>
+      <c r="Q37" s="16"/>
+      <c r="R37" s="16"/>
+      <c r="S37" s="16"/>
+      <c r="T37" s="16"/>
+      <c r="U37" s="16"/>
+      <c r="V37" s="16"/>
+      <c r="W37" s="16"/>
+      <c r="X37" s="16"/>
+      <c r="Y37" s="16"/>
+      <c r="Z37" s="16"/>
+      <c r="AA37" s="16"/>
+      <c r="AB37" s="16"/>
+      <c r="AC37" s="16"/>
+      <c r="AD37" s="16"/>
+      <c r="AE37" s="16"/>
+      <c r="AF37" s="16"/>
+      <c r="AG37" s="16"/>
+      <c r="AH37" s="16"/>
+      <c r="AI37" s="16"/>
+      <c r="AJ37" s="16"/>
+      <c r="AK37" s="16"/>
+      <c r="AL37" s="16"/>
+      <c r="AM37" s="16"/>
+      <c r="AO37" s="16" t="str">
         <f t="shared" si="17"/>
-        <v>-0.0367</v>
-      </c>
-      <c r="F37" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.0146</v>
-      </c>
-      <c r="G37" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.021</v>
-      </c>
-      <c r="H37" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.0463</v>
-      </c>
-      <c r="I37" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.021</v>
-      </c>
-      <c r="J37" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.08</v>
-      </c>
-      <c r="K37" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.016</v>
-      </c>
-      <c r="L37" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.052</v>
-      </c>
-      <c r="M37" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.0003</v>
-      </c>
-      <c r="N37" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.08</v>
-      </c>
-      <c r="O37" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.0571</v>
-      </c>
-      <c r="P37" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.08</v>
-      </c>
-      <c r="Q37" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.0301</v>
-      </c>
-      <c r="R37" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.007</v>
-      </c>
-      <c r="S37" s="16">
-        <f t="shared" si="17"/>
-        <v>0</v>
-      </c>
-      <c r="T37" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.0021</v>
-      </c>
-      <c r="U37" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.0111</v>
-      </c>
-      <c r="V37" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.0782</v>
-      </c>
-      <c r="W37" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.0089</v>
-      </c>
-      <c r="X37" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.0221</v>
-      </c>
-      <c r="Y37" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.0616</v>
-      </c>
-      <c r="Z37" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.0117</v>
-      </c>
-      <c r="AA37" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.0632</v>
-      </c>
-      <c r="AB37" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.08</v>
-      </c>
-      <c r="AC37" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.02</v>
-      </c>
-      <c r="AD37" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.08</v>
-      </c>
-      <c r="AE37" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.0629</v>
-      </c>
-      <c r="AF37" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.0001</v>
-      </c>
-      <c r="AG37" s="16">
-        <f t="shared" si="17"/>
-        <v>-0.0374</v>
-      </c>
-      <c r="AH37" s="16">
+        <v>ELE,CHP</v>
+      </c>
+      <c r="AP37" s="16" t="str">
         <f t="shared" si="13"/>
-        <v>-0.01</v>
-      </c>
-      <c r="AI37" s="16">
-        <f t="shared" si="13"/>
-        <v>-0.026</v>
-      </c>
-      <c r="AJ37" s="16">
-        <f t="shared" si="13"/>
-        <v>-0.0059</v>
-      </c>
-      <c r="AK37" s="16">
-        <f t="shared" si="13"/>
-        <v>-0.022</v>
-      </c>
-      <c r="AL37" s="16">
-        <f t="shared" si="13"/>
-        <v>-0.08</v>
-      </c>
-      <c r="AM37" s="16">
-        <f t="shared" si="13"/>
-        <v>-0.0103</v>
-      </c>
-      <c r="AO37" s="16" t="str">
-        <f t="shared" si="18"/>
-        <v>ELE,CHP</v>
-      </c>
-      <c r="AP37" s="16" t="str">
-        <f t="shared" si="14"/>
         <v>???oil*</v>
       </c>
       <c r="AR37" s="43" t="s">
@@ -27090,19 +26844,17 @@
       </c>
     </row>
     <row r="38" spans="1:46">
-      <c r="A38" s="19">
-        <v>0.1</v>
-      </c>
+      <c r="A38" s="19"/>
       <c r="B38" t="str">
+        <f t="shared" si="14"/>
+        <v>UCE_utilization_bioenergy_UP</v>
+      </c>
+      <c r="C38" t="str">
+        <f t="shared" si="14"/>
+        <v>UP</v>
+      </c>
+      <c r="D38">
         <f t="shared" si="15"/>
-        <v>UCE_utilization_bioenergy_UP</v>
-      </c>
-      <c r="C38" t="str">
-        <f t="shared" si="15"/>
-        <v>UP</v>
-      </c>
-      <c r="D38">
-        <f t="shared" si="16"/>
         <v>2030</v>
       </c>
       <c r="E38" s="20">
@@ -27110,315 +26862,313 @@
         <v>-0.057</v>
       </c>
       <c r="F38" s="20">
-        <f t="shared" ref="F38:AM39" si="19">IF(F12="","",-F12)</f>
+        <f t="shared" ref="F38:AM39" si="18">IF(F12="","",-F12)</f>
         <v>-0.287</v>
       </c>
       <c r="G38" s="20">
+        <f t="shared" si="18"/>
+        <v>-0.506</v>
+      </c>
+      <c r="H38" s="20">
+        <f t="shared" si="18"/>
+        <v>-0.564</v>
+      </c>
+      <c r="I38" s="20">
+        <f t="shared" si="18"/>
+        <v>-0.842</v>
+      </c>
+      <c r="J38" s="20">
+        <f t="shared" si="18"/>
+        <v>-0.95</v>
+      </c>
+      <c r="K38" s="20">
+        <f t="shared" si="18"/>
+        <v>-0.436</v>
+      </c>
+      <c r="L38" s="20">
+        <f t="shared" si="18"/>
+        <v>-0.95</v>
+      </c>
+      <c r="M38" s="20">
+        <f t="shared" si="18"/>
+        <v>-0.711</v>
+      </c>
+      <c r="N38" s="20">
+        <f t="shared" si="18"/>
+        <v>-0.77</v>
+      </c>
+      <c r="O38" s="20">
+        <f t="shared" si="18"/>
+        <v>-0.834</v>
+      </c>
+      <c r="P38" s="20">
+        <f t="shared" si="18"/>
+        <v>-0.769</v>
+      </c>
+      <c r="Q38" s="20">
+        <f t="shared" si="18"/>
+        <v>-0.587</v>
+      </c>
+      <c r="R38" s="20">
+        <f t="shared" si="18"/>
+        <v>-0.879</v>
+      </c>
+      <c r="S38" s="20" t="str">
+        <f t="shared" si="18"/>
+        <v/>
+      </c>
+      <c r="T38" s="20">
+        <f t="shared" si="18"/>
+        <v>-0.655</v>
+      </c>
+      <c r="U38" s="20">
+        <f t="shared" si="18"/>
+        <v>-0.95</v>
+      </c>
+      <c r="V38" s="20">
+        <f t="shared" si="18"/>
+        <v>-0.751</v>
+      </c>
+      <c r="W38" s="20">
+        <f t="shared" si="18"/>
+        <v>-0.95</v>
+      </c>
+      <c r="X38" s="20">
+        <f t="shared" si="18"/>
+        <v>-0.462</v>
+      </c>
+      <c r="Y38" s="20">
+        <f t="shared" si="18"/>
+        <v>-0.95</v>
+      </c>
+      <c r="Z38" s="20">
+        <f t="shared" si="18"/>
+        <v>-0.644</v>
+      </c>
+      <c r="AA38" s="20">
+        <f t="shared" si="18"/>
+        <v>-0.95</v>
+      </c>
+      <c r="AB38" s="20">
+        <f t="shared" si="18"/>
+        <v>-0.95</v>
+      </c>
+      <c r="AC38" s="20">
+        <f t="shared" si="18"/>
+        <v>-0.564</v>
+      </c>
+      <c r="AD38" s="20">
+        <f t="shared" si="18"/>
+        <v>-0.107</v>
+      </c>
+      <c r="AE38" s="20" t="str">
+        <f t="shared" si="18"/>
+        <v/>
+      </c>
+      <c r="AF38" s="20">
+        <f t="shared" si="18"/>
+        <v>-0.189</v>
+      </c>
+      <c r="AG38" s="20">
+        <f t="shared" si="18"/>
+        <v>-0.727</v>
+      </c>
+      <c r="AH38" s="20">
+        <f t="shared" si="18"/>
+        <v>-0.476</v>
+      </c>
+      <c r="AI38" s="20">
+        <f t="shared" si="18"/>
+        <v>-0.95</v>
+      </c>
+      <c r="AJ38" s="20">
+        <f t="shared" si="18"/>
+        <v>-0.56</v>
+      </c>
+      <c r="AK38" s="20">
+        <f t="shared" si="18"/>
+        <v>-0.77</v>
+      </c>
+      <c r="AL38" s="20">
+        <f t="shared" si="18"/>
+        <v>-0.41</v>
+      </c>
+      <c r="AM38" s="20">
+        <f t="shared" si="18"/>
+        <v>-0.95</v>
+      </c>
+      <c r="AO38" s="16" t="str">
+        <f t="shared" si="17"/>
+        <v>ELE,CHP</v>
+      </c>
+      <c r="AP38" s="16" t="str">
+        <f t="shared" si="13"/>
+        <v>elcbsl,indbio</v>
+      </c>
+      <c r="AR38" s="43" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="39" spans="1:46">
+      <c r="A39" s="19"/>
+      <c r="B39" t="str">
+        <f t="shared" si="14"/>
+        <v>UCE_utilization_coal_UP</v>
+      </c>
+      <c r="C39" t="str">
+        <f t="shared" si="14"/>
+        <v>UP</v>
+      </c>
+      <c r="D39">
+        <f t="shared" si="15"/>
+        <v>2030</v>
+      </c>
+      <c r="E39" s="20">
+        <f t="shared" ref="E39:AG39" si="19">IF(E13="","",-E13)</f>
+        <v>-0.777</v>
+      </c>
+      <c r="F39" s="20">
         <f t="shared" si="19"/>
-        <v>-0.506</v>
-      </c>
-      <c r="H38" s="20">
+        <v>-0.47</v>
+      </c>
+      <c r="G39" s="20">
         <f t="shared" si="19"/>
-        <v>-0.564</v>
-      </c>
-      <c r="I38" s="20">
-        <f t="shared" si="19"/>
-        <v>-0.842</v>
-      </c>
-      <c r="J38" s="20">
+        <v>-0.724</v>
+      </c>
+      <c r="H39" s="20">
         <f t="shared" si="19"/>
         <v>-0.95</v>
       </c>
-      <c r="K38" s="20">
-        <f t="shared" si="19"/>
-        <v>-0.436</v>
-      </c>
-      <c r="L38" s="20">
+      <c r="I39" s="20">
         <f t="shared" si="19"/>
         <v>-0.95</v>
       </c>
-      <c r="M38" s="20">
+      <c r="J39" s="20">
         <f t="shared" si="19"/>
-        <v>-0.711</v>
-      </c>
-      <c r="N38" s="20">
+        <v>-0.95</v>
+      </c>
+      <c r="K39" s="20">
         <f t="shared" si="19"/>
-        <v>-0.77</v>
-      </c>
-      <c r="O38" s="20">
-        <f t="shared" si="19"/>
-        <v>-0.834</v>
-      </c>
-      <c r="P38" s="20">
-        <f t="shared" si="19"/>
-        <v>-0.769</v>
-      </c>
-      <c r="Q38" s="20">
+        <v>-0.922</v>
+      </c>
+      <c r="L39" s="20">
         <f t="shared" si="19"/>
         <v>-0.587</v>
       </c>
-      <c r="R38" s="20">
+      <c r="M39" s="20">
         <f t="shared" si="19"/>
-        <v>-0.879</v>
-      </c>
-      <c r="S38" s="20" t="str">
+        <v>-0.578</v>
+      </c>
+      <c r="N39" s="20">
+        <f t="shared" si="19"/>
+        <v>-0.544</v>
+      </c>
+      <c r="O39" s="20">
+        <f t="shared" si="19"/>
+        <v>-0.391</v>
+      </c>
+      <c r="P39" s="20">
+        <f t="shared" si="19"/>
+        <v>-0.625</v>
+      </c>
+      <c r="Q39" s="20">
+        <f t="shared" si="19"/>
+        <v>-0.597</v>
+      </c>
+      <c r="R39" s="20">
+        <f t="shared" si="19"/>
+        <v>-0.431</v>
+      </c>
+      <c r="S39" s="20" t="str">
         <f t="shared" si="19"/>
         <v/>
       </c>
-      <c r="T38" s="20">
+      <c r="T39" s="20">
         <f t="shared" si="19"/>
-        <v>-0.655</v>
-      </c>
-      <c r="U38" s="20">
+        <v>-0.707</v>
+      </c>
+      <c r="U39" s="20">
+        <f t="shared" si="19"/>
+        <v>-0.604</v>
+      </c>
+      <c r="V39" s="20">
+        <f t="shared" si="19"/>
+        <v>-0.509</v>
+      </c>
+      <c r="W39" s="20">
+        <f t="shared" si="19"/>
+        <v>-0.9</v>
+      </c>
+      <c r="X39" s="20">
+        <f t="shared" si="19"/>
+        <v>-0.777</v>
+      </c>
+      <c r="Y39" s="20">
         <f t="shared" si="19"/>
         <v>-0.95</v>
       </c>
-      <c r="V38" s="20">
+      <c r="Z39" s="20">
         <f t="shared" si="19"/>
-        <v>-0.751</v>
-      </c>
-      <c r="W38" s="20">
+        <v>-0.568</v>
+      </c>
+      <c r="AA39" s="20">
         <f t="shared" si="19"/>
         <v>-0.95</v>
       </c>
-      <c r="X38" s="20">
+      <c r="AB39" s="20">
         <f t="shared" si="19"/>
-        <v>-0.462</v>
-      </c>
-      <c r="Y38" s="20">
+        <v>-0.522</v>
+      </c>
+      <c r="AC39" s="20">
         <f t="shared" si="19"/>
-        <v>-0.95</v>
-      </c>
-      <c r="Z38" s="20">
+        <v>-0.7</v>
+      </c>
+      <c r="AD39" s="20">
         <f t="shared" si="19"/>
-        <v>-0.644</v>
-      </c>
-      <c r="AA38" s="20">
-        <f t="shared" si="19"/>
-        <v>-0.95</v>
-      </c>
-      <c r="AB38" s="20">
-        <f t="shared" si="19"/>
-        <v>-0.95</v>
-      </c>
-      <c r="AC38" s="20">
-        <f t="shared" si="19"/>
-        <v>-0.564</v>
-      </c>
-      <c r="AD38" s="20">
-        <f t="shared" si="19"/>
-        <v>-0.107</v>
-      </c>
-      <c r="AE38" s="20" t="str">
+        <v>-0.637</v>
+      </c>
+      <c r="AE39" s="20" t="str">
         <f t="shared" si="19"/>
         <v/>
       </c>
-      <c r="AF38" s="20">
+      <c r="AF39" s="20">
         <f t="shared" si="19"/>
-        <v>-0.189</v>
-      </c>
-      <c r="AG38" s="20">
+        <v>-0.671</v>
+      </c>
+      <c r="AG39" s="20">
         <f t="shared" si="19"/>
-        <v>-0.727</v>
-      </c>
-      <c r="AH38" s="20">
-        <f t="shared" si="19"/>
-        <v>-0.476</v>
-      </c>
-      <c r="AI38" s="20">
-        <f t="shared" si="19"/>
-        <v>-0.95</v>
-      </c>
-      <c r="AJ38" s="20">
-        <f t="shared" si="19"/>
-        <v>-0.56</v>
-      </c>
-      <c r="AK38" s="20">
-        <f t="shared" si="19"/>
-        <v>-0.77</v>
-      </c>
-      <c r="AL38" s="20">
-        <f t="shared" si="19"/>
-        <v>-0.41</v>
-      </c>
-      <c r="AM38" s="20">
-        <f t="shared" si="19"/>
-        <v>-0.95</v>
-      </c>
-      <c r="AO38" s="16" t="str">
+        <v>-0.575</v>
+      </c>
+      <c r="AH39" s="20">
         <f t="shared" si="18"/>
+        <v>-0.351</v>
+      </c>
+      <c r="AI39" s="20" t="str">
+        <f t="shared" si="18"/>
+        <v/>
+      </c>
+      <c r="AJ39" s="20">
+        <f t="shared" si="18"/>
+        <v>-0.679</v>
+      </c>
+      <c r="AK39" s="20">
+        <f t="shared" si="18"/>
+        <v>-0.539</v>
+      </c>
+      <c r="AL39" s="20">
+        <f t="shared" si="18"/>
+        <v>-0.319</v>
+      </c>
+      <c r="AM39" s="20">
+        <f t="shared" si="18"/>
+        <v>-0.695</v>
+      </c>
+      <c r="AO39" s="16" t="str">
+        <f t="shared" si="17"/>
         <v>ELE,CHP</v>
       </c>
-      <c r="AP38" s="16" t="str">
-        <f t="shared" si="14"/>
-        <v>elcbsl,indbio</v>
-      </c>
-      <c r="AR38" s="43" t="s">
-        <v>341</v>
-      </c>
-    </row>
-    <row r="39" spans="1:46">
-      <c r="A39" s="19">
-        <v>0.1</v>
-      </c>
-      <c r="B39" t="str">
-        <f t="shared" si="15"/>
-        <v>UCE_utilization_coal_UP</v>
-      </c>
-      <c r="C39" t="str">
-        <f t="shared" si="15"/>
-        <v>UP</v>
-      </c>
-      <c r="D39">
-        <f t="shared" si="16"/>
-        <v>2030</v>
-      </c>
-      <c r="E39" s="20">
-        <f t="shared" ref="E39:AG39" si="20">IF(E13="","",-E13)</f>
-        <v>-0.777</v>
-      </c>
-      <c r="F39" s="20">
-        <f t="shared" si="20"/>
-        <v>-0.47</v>
-      </c>
-      <c r="G39" s="20">
-        <f t="shared" si="20"/>
-        <v>-0.724</v>
-      </c>
-      <c r="H39" s="20">
-        <f t="shared" si="20"/>
-        <v>-0.95</v>
-      </c>
-      <c r="I39" s="20">
-        <f t="shared" si="20"/>
-        <v>-0.95</v>
-      </c>
-      <c r="J39" s="20">
-        <f t="shared" si="20"/>
-        <v>-0.95</v>
-      </c>
-      <c r="K39" s="20">
-        <f t="shared" si="20"/>
-        <v>-0.922</v>
-      </c>
-      <c r="L39" s="20">
-        <f t="shared" si="20"/>
-        <v>-0.587</v>
-      </c>
-      <c r="M39" s="20">
-        <f t="shared" si="20"/>
-        <v>-0.578</v>
-      </c>
-      <c r="N39" s="20">
-        <f t="shared" si="20"/>
-        <v>-0.544</v>
-      </c>
-      <c r="O39" s="20">
-        <f t="shared" si="20"/>
-        <v>-0.391</v>
-      </c>
-      <c r="P39" s="20">
-        <f t="shared" si="20"/>
-        <v>-0.625</v>
-      </c>
-      <c r="Q39" s="20">
-        <f t="shared" si="20"/>
-        <v>-0.597</v>
-      </c>
-      <c r="R39" s="20">
-        <f t="shared" si="20"/>
-        <v>-0.431</v>
-      </c>
-      <c r="S39" s="20" t="str">
-        <f t="shared" si="20"/>
-        <v/>
-      </c>
-      <c r="T39" s="20">
-        <f t="shared" si="20"/>
-        <v>-0.707</v>
-      </c>
-      <c r="U39" s="20">
-        <f t="shared" si="20"/>
-        <v>-0.604</v>
-      </c>
-      <c r="V39" s="20">
-        <f t="shared" si="20"/>
-        <v>-0.509</v>
-      </c>
-      <c r="W39" s="20">
-        <f t="shared" si="20"/>
-        <v>-0.9</v>
-      </c>
-      <c r="X39" s="20">
-        <f t="shared" si="20"/>
-        <v>-0.777</v>
-      </c>
-      <c r="Y39" s="20">
-        <f t="shared" si="20"/>
-        <v>-0.95</v>
-      </c>
-      <c r="Z39" s="20">
-        <f t="shared" si="20"/>
-        <v>-0.568</v>
-      </c>
-      <c r="AA39" s="20">
-        <f t="shared" si="20"/>
-        <v>-0.95</v>
-      </c>
-      <c r="AB39" s="20">
-        <f t="shared" si="20"/>
-        <v>-0.522</v>
-      </c>
-      <c r="AC39" s="20">
-        <f t="shared" si="20"/>
-        <v>-0.7</v>
-      </c>
-      <c r="AD39" s="20">
-        <f t="shared" si="20"/>
-        <v>-0.637</v>
-      </c>
-      <c r="AE39" s="20" t="str">
-        <f t="shared" si="20"/>
-        <v/>
-      </c>
-      <c r="AF39" s="20">
-        <f t="shared" si="20"/>
-        <v>-0.671</v>
-      </c>
-      <c r="AG39" s="20">
-        <f t="shared" si="20"/>
-        <v>-0.575</v>
-      </c>
-      <c r="AH39" s="20">
-        <f t="shared" si="19"/>
-        <v>-0.351</v>
-      </c>
-      <c r="AI39" s="20" t="str">
-        <f t="shared" si="19"/>
-        <v/>
-      </c>
-      <c r="AJ39" s="20">
-        <f t="shared" si="19"/>
-        <v>-0.679</v>
-      </c>
-      <c r="AK39" s="20">
-        <f t="shared" si="19"/>
-        <v>-0.539</v>
-      </c>
-      <c r="AL39" s="20">
-        <f t="shared" si="19"/>
-        <v>-0.319</v>
-      </c>
-      <c r="AM39" s="20">
-        <f t="shared" si="19"/>
-        <v>-0.695</v>
-      </c>
-      <c r="AO39" s="16" t="str">
-        <f t="shared" si="18"/>
-        <v>ELE,CHP</v>
-      </c>
       <c r="AP39" s="16" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>???coa,elccob</v>
       </c>
       <c r="AR39" s="43" t="s">
@@ -27430,15 +27180,15 @@
         <v>0.8</v>
       </c>
       <c r="B40" t="str">
+        <f t="shared" si="14"/>
+        <v>UCE_utilization_gas_UP</v>
+      </c>
+      <c r="C40" t="str">
+        <f t="shared" si="14"/>
+        <v>UP</v>
+      </c>
+      <c r="D40">
         <f t="shared" si="15"/>
-        <v>UCE_utilization_gas_UP</v>
-      </c>
-      <c r="C40" t="str">
-        <f t="shared" si="15"/>
-        <v>UP</v>
-      </c>
-      <c r="D40">
-        <f t="shared" si="16"/>
         <v>2030</v>
       </c>
       <c r="E40">
@@ -27446,147 +27196,147 @@
         <v>-0.8</v>
       </c>
       <c r="F40">
-        <f t="shared" ref="F40:U42" si="21">-$A40</f>
+        <f t="shared" ref="F40:U42" si="20">-$A40</f>
         <v>-0.8</v>
       </c>
       <c r="G40">
+        <f t="shared" si="20"/>
+        <v>-0.8</v>
+      </c>
+      <c r="H40">
+        <f t="shared" si="20"/>
+        <v>-0.8</v>
+      </c>
+      <c r="I40">
+        <f t="shared" si="20"/>
+        <v>-0.8</v>
+      </c>
+      <c r="J40">
+        <f t="shared" si="20"/>
+        <v>-0.8</v>
+      </c>
+      <c r="K40">
+        <f t="shared" si="20"/>
+        <v>-0.8</v>
+      </c>
+      <c r="L40">
+        <f t="shared" si="20"/>
+        <v>-0.8</v>
+      </c>
+      <c r="M40">
+        <f t="shared" si="20"/>
+        <v>-0.8</v>
+      </c>
+      <c r="N40">
+        <f t="shared" si="20"/>
+        <v>-0.8</v>
+      </c>
+      <c r="O40">
+        <f t="shared" si="20"/>
+        <v>-0.8</v>
+      </c>
+      <c r="P40">
+        <f t="shared" si="20"/>
+        <v>-0.8</v>
+      </c>
+      <c r="Q40">
+        <f t="shared" si="20"/>
+        <v>-0.8</v>
+      </c>
+      <c r="R40">
+        <f t="shared" si="20"/>
+        <v>-0.8</v>
+      </c>
+      <c r="S40">
+        <f t="shared" si="20"/>
+        <v>-0.8</v>
+      </c>
+      <c r="T40">
+        <f t="shared" si="20"/>
+        <v>-0.8</v>
+      </c>
+      <c r="U40">
+        <f t="shared" si="20"/>
+        <v>-0.8</v>
+      </c>
+      <c r="V40">
+        <f t="shared" ref="V40:AK42" si="21">-$A40</f>
+        <v>-0.8</v>
+      </c>
+      <c r="W40">
         <f t="shared" si="21"/>
         <v>-0.8</v>
       </c>
-      <c r="H40">
+      <c r="X40">
         <f t="shared" si="21"/>
         <v>-0.8</v>
       </c>
-      <c r="I40">
+      <c r="Y40">
         <f t="shared" si="21"/>
         <v>-0.8</v>
       </c>
-      <c r="J40">
+      <c r="Z40">
         <f t="shared" si="21"/>
         <v>-0.8</v>
       </c>
-      <c r="K40">
+      <c r="AA40">
         <f t="shared" si="21"/>
         <v>-0.8</v>
       </c>
-      <c r="L40">
+      <c r="AB40">
         <f t="shared" si="21"/>
         <v>-0.8</v>
       </c>
-      <c r="M40">
+      <c r="AC40">
         <f t="shared" si="21"/>
         <v>-0.8</v>
       </c>
-      <c r="N40">
+      <c r="AD40">
         <f t="shared" si="21"/>
         <v>-0.8</v>
       </c>
-      <c r="O40">
+      <c r="AE40">
         <f t="shared" si="21"/>
         <v>-0.8</v>
       </c>
-      <c r="P40">
+      <c r="AF40">
         <f t="shared" si="21"/>
         <v>-0.8</v>
       </c>
-      <c r="Q40">
+      <c r="AG40">
         <f t="shared" si="21"/>
         <v>-0.8</v>
       </c>
-      <c r="R40">
+      <c r="AH40">
         <f t="shared" si="21"/>
         <v>-0.8</v>
       </c>
-      <c r="S40">
+      <c r="AI40">
         <f t="shared" si="21"/>
         <v>-0.8</v>
       </c>
-      <c r="T40">
+      <c r="AJ40">
         <f t="shared" si="21"/>
         <v>-0.8</v>
       </c>
-      <c r="U40">
+      <c r="AK40">
         <f t="shared" si="21"/>
         <v>-0.8</v>
       </c>
-      <c r="V40">
-        <f t="shared" ref="V40:AK42" si="22">-$A40</f>
+      <c r="AL40">
+        <f t="shared" ref="AL40:AM42" si="22">-$A40</f>
         <v>-0.8</v>
       </c>
-      <c r="W40">
+      <c r="AM40">
         <f t="shared" si="22"/>
         <v>-0.8</v>
       </c>
-      <c r="X40">
-        <f t="shared" si="22"/>
-        <v>-0.8</v>
-      </c>
-      <c r="Y40">
-        <f t="shared" si="22"/>
-        <v>-0.8</v>
-      </c>
-      <c r="Z40">
-        <f t="shared" si="22"/>
-        <v>-0.8</v>
-      </c>
-      <c r="AA40">
-        <f t="shared" si="22"/>
-        <v>-0.8</v>
-      </c>
-      <c r="AB40">
-        <f t="shared" si="22"/>
-        <v>-0.8</v>
-      </c>
-      <c r="AC40">
-        <f t="shared" si="22"/>
-        <v>-0.8</v>
-      </c>
-      <c r="AD40">
-        <f t="shared" si="22"/>
-        <v>-0.8</v>
-      </c>
-      <c r="AE40">
-        <f t="shared" si="22"/>
-        <v>-0.8</v>
-      </c>
-      <c r="AF40">
-        <f t="shared" si="22"/>
-        <v>-0.8</v>
-      </c>
-      <c r="AG40">
-        <f t="shared" si="22"/>
-        <v>-0.8</v>
-      </c>
-      <c r="AH40">
-        <f t="shared" si="22"/>
-        <v>-0.8</v>
-      </c>
-      <c r="AI40">
-        <f t="shared" si="22"/>
-        <v>-0.8</v>
-      </c>
-      <c r="AJ40">
-        <f t="shared" si="22"/>
-        <v>-0.8</v>
-      </c>
-      <c r="AK40">
-        <f t="shared" si="22"/>
-        <v>-0.8</v>
-      </c>
-      <c r="AL40">
-        <f t="shared" ref="AL40:AM42" si="23">-$A40</f>
-        <v>-0.8</v>
-      </c>
-      <c r="AM40">
-        <f t="shared" si="23"/>
-        <v>-0.8</v>
-      </c>
       <c r="AO40" s="16" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="17"/>
         <v>ELE,CHP</v>
       </c>
       <c r="AP40" s="16" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>???nga</v>
       </c>
       <c r="AR40" s="43" t="s">
@@ -27598,163 +27348,163 @@
         <v>0.95</v>
       </c>
       <c r="B41" t="str">
+        <f t="shared" si="14"/>
+        <v>UCE_utilization_nuclear_UP</v>
+      </c>
+      <c r="C41" t="str">
+        <f t="shared" si="14"/>
+        <v>UP</v>
+      </c>
+      <c r="D41">
         <f t="shared" si="15"/>
-        <v>UCE_utilization_nuclear_UP</v>
-      </c>
-      <c r="C41" t="str">
-        <f t="shared" si="15"/>
-        <v>UP</v>
-      </c>
-      <c r="D41">
-        <f t="shared" si="16"/>
         <v>2030</v>
       </c>
       <c r="E41">
-        <f t="shared" ref="E41:E42" si="24">-$A41</f>
+        <f t="shared" ref="E41:E42" si="23">-$A41</f>
         <v>-0.95</v>
       </c>
       <c r="F41">
+        <f t="shared" si="20"/>
+        <v>-0.95</v>
+      </c>
+      <c r="G41">
+        <f t="shared" si="20"/>
+        <v>-0.95</v>
+      </c>
+      <c r="H41">
+        <f t="shared" si="20"/>
+        <v>-0.95</v>
+      </c>
+      <c r="I41">
+        <f t="shared" si="20"/>
+        <v>-0.95</v>
+      </c>
+      <c r="J41">
+        <f t="shared" si="20"/>
+        <v>-0.95</v>
+      </c>
+      <c r="K41">
+        <f t="shared" si="20"/>
+        <v>-0.95</v>
+      </c>
+      <c r="L41">
+        <f t="shared" si="20"/>
+        <v>-0.95</v>
+      </c>
+      <c r="M41">
+        <f t="shared" si="20"/>
+        <v>-0.95</v>
+      </c>
+      <c r="N41">
+        <f t="shared" si="20"/>
+        <v>-0.95</v>
+      </c>
+      <c r="O41">
+        <f t="shared" si="20"/>
+        <v>-0.95</v>
+      </c>
+      <c r="P41">
+        <f t="shared" si="20"/>
+        <v>-0.95</v>
+      </c>
+      <c r="Q41">
+        <f t="shared" si="20"/>
+        <v>-0.95</v>
+      </c>
+      <c r="R41">
+        <f t="shared" si="20"/>
+        <v>-0.95</v>
+      </c>
+      <c r="S41">
+        <f t="shared" si="20"/>
+        <v>-0.95</v>
+      </c>
+      <c r="T41">
+        <f t="shared" si="20"/>
+        <v>-0.95</v>
+      </c>
+      <c r="U41">
+        <f t="shared" si="20"/>
+        <v>-0.95</v>
+      </c>
+      <c r="V41">
         <f t="shared" si="21"/>
         <v>-0.95</v>
       </c>
-      <c r="G41">
+      <c r="W41">
         <f t="shared" si="21"/>
         <v>-0.95</v>
       </c>
-      <c r="H41">
+      <c r="X41">
         <f t="shared" si="21"/>
         <v>-0.95</v>
       </c>
-      <c r="I41">
+      <c r="Y41">
         <f t="shared" si="21"/>
         <v>-0.95</v>
       </c>
-      <c r="J41">
+      <c r="Z41">
         <f t="shared" si="21"/>
         <v>-0.95</v>
       </c>
-      <c r="K41">
+      <c r="AA41">
         <f t="shared" si="21"/>
         <v>-0.95</v>
       </c>
-      <c r="L41">
+      <c r="AB41">
         <f t="shared" si="21"/>
         <v>-0.95</v>
       </c>
-      <c r="M41">
+      <c r="AC41">
         <f t="shared" si="21"/>
         <v>-0.95</v>
       </c>
-      <c r="N41">
+      <c r="AD41">
         <f t="shared" si="21"/>
         <v>-0.95</v>
       </c>
-      <c r="O41">
+      <c r="AE41">
         <f t="shared" si="21"/>
         <v>-0.95</v>
       </c>
-      <c r="P41">
+      <c r="AF41">
         <f t="shared" si="21"/>
         <v>-0.95</v>
       </c>
-      <c r="Q41">
+      <c r="AG41">
         <f t="shared" si="21"/>
         <v>-0.95</v>
       </c>
-      <c r="R41">
+      <c r="AH41">
         <f t="shared" si="21"/>
         <v>-0.95</v>
       </c>
-      <c r="S41">
+      <c r="AI41">
         <f t="shared" si="21"/>
         <v>-0.95</v>
       </c>
-      <c r="T41">
+      <c r="AJ41">
         <f t="shared" si="21"/>
         <v>-0.95</v>
       </c>
-      <c r="U41">
+      <c r="AK41">
         <f t="shared" si="21"/>
         <v>-0.95</v>
       </c>
-      <c r="V41">
+      <c r="AL41">
         <f t="shared" si="22"/>
         <v>-0.95</v>
       </c>
-      <c r="W41">
+      <c r="AM41">
         <f t="shared" si="22"/>
         <v>-0.95</v>
       </c>
-      <c r="X41">
-        <f t="shared" si="22"/>
-        <v>-0.95</v>
-      </c>
-      <c r="Y41">
-        <f t="shared" si="22"/>
-        <v>-0.95</v>
-      </c>
-      <c r="Z41">
-        <f t="shared" si="22"/>
-        <v>-0.95</v>
-      </c>
-      <c r="AA41">
-        <f t="shared" si="22"/>
-        <v>-0.95</v>
-      </c>
-      <c r="AB41">
-        <f t="shared" si="22"/>
-        <v>-0.95</v>
-      </c>
-      <c r="AC41">
-        <f t="shared" si="22"/>
-        <v>-0.95</v>
-      </c>
-      <c r="AD41">
-        <f t="shared" si="22"/>
-        <v>-0.95</v>
-      </c>
-      <c r="AE41">
-        <f t="shared" si="22"/>
-        <v>-0.95</v>
-      </c>
-      <c r="AF41">
-        <f t="shared" si="22"/>
-        <v>-0.95</v>
-      </c>
-      <c r="AG41">
-        <f t="shared" si="22"/>
-        <v>-0.95</v>
-      </c>
-      <c r="AH41">
-        <f t="shared" si="22"/>
-        <v>-0.95</v>
-      </c>
-      <c r="AI41">
-        <f t="shared" si="22"/>
-        <v>-0.95</v>
-      </c>
-      <c r="AJ41">
-        <f t="shared" si="22"/>
-        <v>-0.95</v>
-      </c>
-      <c r="AK41">
-        <f t="shared" si="22"/>
-        <v>-0.95</v>
-      </c>
-      <c r="AL41">
-        <f t="shared" si="23"/>
-        <v>-0.95</v>
-      </c>
-      <c r="AM41">
-        <f t="shared" si="23"/>
-        <v>-0.95</v>
-      </c>
       <c r="AO41" s="16" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="17"/>
         <v>ELE,CHP</v>
       </c>
       <c r="AP41" s="16" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>???nuc</v>
       </c>
       <c r="AR41" s="43" t="s">
@@ -27766,163 +27516,163 @@
         <v>0.8</v>
       </c>
       <c r="B42" t="str">
+        <f t="shared" si="14"/>
+        <v>UCE_utilization_oil_UP</v>
+      </c>
+      <c r="C42" t="str">
+        <f t="shared" si="14"/>
+        <v>UP</v>
+      </c>
+      <c r="D42">
         <f t="shared" si="15"/>
-        <v>UCE_utilization_oil_UP</v>
-      </c>
-      <c r="C42" t="str">
-        <f t="shared" si="15"/>
-        <v>UP</v>
-      </c>
-      <c r="D42">
-        <f t="shared" si="16"/>
         <v>2030</v>
       </c>
       <c r="E42">
-        <f t="shared" si="24"/>
+        <f t="shared" si="23"/>
         <v>-0.8</v>
       </c>
       <c r="F42">
+        <f t="shared" si="20"/>
+        <v>-0.8</v>
+      </c>
+      <c r="G42">
+        <f t="shared" si="20"/>
+        <v>-0.8</v>
+      </c>
+      <c r="H42">
+        <f t="shared" si="20"/>
+        <v>-0.8</v>
+      </c>
+      <c r="I42">
+        <f t="shared" si="20"/>
+        <v>-0.8</v>
+      </c>
+      <c r="J42">
+        <f t="shared" si="20"/>
+        <v>-0.8</v>
+      </c>
+      <c r="K42">
+        <f t="shared" si="20"/>
+        <v>-0.8</v>
+      </c>
+      <c r="L42">
+        <f t="shared" si="20"/>
+        <v>-0.8</v>
+      </c>
+      <c r="M42">
+        <f t="shared" si="20"/>
+        <v>-0.8</v>
+      </c>
+      <c r="N42">
+        <f t="shared" si="20"/>
+        <v>-0.8</v>
+      </c>
+      <c r="O42">
+        <f t="shared" si="20"/>
+        <v>-0.8</v>
+      </c>
+      <c r="P42">
+        <f t="shared" si="20"/>
+        <v>-0.8</v>
+      </c>
+      <c r="Q42">
+        <f t="shared" si="20"/>
+        <v>-0.8</v>
+      </c>
+      <c r="R42">
+        <f t="shared" si="20"/>
+        <v>-0.8</v>
+      </c>
+      <c r="S42">
+        <f t="shared" si="20"/>
+        <v>-0.8</v>
+      </c>
+      <c r="T42">
+        <f t="shared" si="20"/>
+        <v>-0.8</v>
+      </c>
+      <c r="U42">
+        <f t="shared" si="20"/>
+        <v>-0.8</v>
+      </c>
+      <c r="V42">
         <f t="shared" si="21"/>
         <v>-0.8</v>
       </c>
-      <c r="G42">
+      <c r="W42">
         <f t="shared" si="21"/>
         <v>-0.8</v>
       </c>
-      <c r="H42">
+      <c r="X42">
         <f t="shared" si="21"/>
         <v>-0.8</v>
       </c>
-      <c r="I42">
+      <c r="Y42">
         <f t="shared" si="21"/>
         <v>-0.8</v>
       </c>
-      <c r="J42">
+      <c r="Z42">
         <f t="shared" si="21"/>
         <v>-0.8</v>
       </c>
-      <c r="K42">
+      <c r="AA42">
         <f t="shared" si="21"/>
         <v>-0.8</v>
       </c>
-      <c r="L42">
+      <c r="AB42">
         <f t="shared" si="21"/>
         <v>-0.8</v>
       </c>
-      <c r="M42">
+      <c r="AC42">
         <f t="shared" si="21"/>
         <v>-0.8</v>
       </c>
-      <c r="N42">
+      <c r="AD42">
         <f t="shared" si="21"/>
         <v>-0.8</v>
       </c>
-      <c r="O42">
+      <c r="AE42">
         <f t="shared" si="21"/>
         <v>-0.8</v>
       </c>
-      <c r="P42">
+      <c r="AF42">
         <f t="shared" si="21"/>
         <v>-0.8</v>
       </c>
-      <c r="Q42">
+      <c r="AG42">
         <f t="shared" si="21"/>
         <v>-0.8</v>
       </c>
-      <c r="R42">
+      <c r="AH42">
         <f t="shared" si="21"/>
         <v>-0.8</v>
       </c>
-      <c r="S42">
+      <c r="AI42">
         <f t="shared" si="21"/>
         <v>-0.8</v>
       </c>
-      <c r="T42">
+      <c r="AJ42">
         <f t="shared" si="21"/>
         <v>-0.8</v>
       </c>
-      <c r="U42">
+      <c r="AK42">
         <f t="shared" si="21"/>
         <v>-0.8</v>
       </c>
-      <c r="V42">
+      <c r="AL42">
         <f t="shared" si="22"/>
         <v>-0.8</v>
       </c>
-      <c r="W42">
+      <c r="AM42">
         <f t="shared" si="22"/>
         <v>-0.8</v>
       </c>
-      <c r="X42">
-        <f t="shared" si="22"/>
-        <v>-0.8</v>
-      </c>
-      <c r="Y42">
-        <f t="shared" si="22"/>
-        <v>-0.8</v>
-      </c>
-      <c r="Z42">
-        <f t="shared" si="22"/>
-        <v>-0.8</v>
-      </c>
-      <c r="AA42">
-        <f t="shared" si="22"/>
-        <v>-0.8</v>
-      </c>
-      <c r="AB42">
-        <f t="shared" si="22"/>
-        <v>-0.8</v>
-      </c>
-      <c r="AC42">
-        <f t="shared" si="22"/>
-        <v>-0.8</v>
-      </c>
-      <c r="AD42">
-        <f t="shared" si="22"/>
-        <v>-0.8</v>
-      </c>
-      <c r="AE42">
-        <f t="shared" si="22"/>
-        <v>-0.8</v>
-      </c>
-      <c r="AF42">
-        <f t="shared" si="22"/>
-        <v>-0.8</v>
-      </c>
-      <c r="AG42">
-        <f t="shared" si="22"/>
-        <v>-0.8</v>
-      </c>
-      <c r="AH42">
-        <f t="shared" si="22"/>
-        <v>-0.8</v>
-      </c>
-      <c r="AI42">
-        <f t="shared" si="22"/>
-        <v>-0.8</v>
-      </c>
-      <c r="AJ42">
-        <f t="shared" si="22"/>
-        <v>-0.8</v>
-      </c>
-      <c r="AK42">
-        <f t="shared" si="22"/>
-        <v>-0.8</v>
-      </c>
-      <c r="AL42">
-        <f t="shared" si="23"/>
-        <v>-0.8</v>
-      </c>
-      <c r="AM42">
-        <f t="shared" si="23"/>
-        <v>-0.8</v>
-      </c>
       <c r="AO42" s="16" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="17"/>
         <v>ELE,CHP</v>
       </c>
       <c r="AP42" s="16" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>???oil*</v>
       </c>
       <c r="AR42" s="43" t="s">
@@ -27932,7 +27682,6 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>
-  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 

</xml_diff>